<commit_message>
guarda index css e imagenes
</commit_message>
<xml_diff>
--- a/excel/preoperacional.xlsx
+++ b/excel/preoperacional.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L189"/>
+  <dimension ref="A1:L214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11198,6 +11198,1431 @@
         </is>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>888888</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Llanta trasera</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>888888</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Llanta delantera</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>888888</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Luces</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>888888</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Direccionales</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>888888</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Motor</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>888888</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Cadena</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>888888</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Freno delantero</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>888888</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Freno trasero</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>888888</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Pedal cambios</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>888888</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Embrague</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>888888</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Tablero</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>888888</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>88888</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Bocina</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Tamayo Camacho</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>15521960</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LLL69A</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>20200</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Llanta trasera</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Tamayo Camacho</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>15521960</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LLL69A</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>20200</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>Llanta delantera</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Tamayo Camacho</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>1111111111</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>HHH22F</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>21411</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Automática</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>Llanta trasera</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Tamayo Camacho</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>1111111111</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>HHH22F</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>21411</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Automática</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>Llanta delantera</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Tamayo Camacho</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>1111111111</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>HHH22F</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>21411</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Automática</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Luces</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Tamayo Camacho</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>1111111111</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>HHH22F</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>21411</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Automática</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Direccionales</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Tamayo Camacho</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>1111111111</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>HHH22F</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>21411</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Automática</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Motor</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Tamayo Camacho</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>1111111111</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>HHH22F</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>21411</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Automática</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Freno delantero</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Tamayo Camacho</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>1111111111</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>HHH22F</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>21411</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Automática</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Freno trasero</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Tamayo Camacho</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>1111111111</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>HHH22F</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>21411</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>Automática</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>Transmisión CVT</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Tamayo Camacho</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>1111111111</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>HHH22F</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>21411</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>Automática</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>Acelerador</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Tamayo Camacho</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>1111111111</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>HHH22F</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>21411</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Automática</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>Tablero</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Tamayo Camacho</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>1111111111</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>HHH22F</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>21411</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Automática</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>Bocina</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Se corrige Google Sheets y mejoras inspeccion
</commit_message>
<xml_diff>
--- a/excel/preoperacional.xlsx
+++ b/excel/preoperacional.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2358,6 +2358,690 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>NWJ76F</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Llanta trasera</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>NWJ76F</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Llanta delantera</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>NWJ76F</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Llanta delantera</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>NWJ76F</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Direccionales</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>NWJ76F</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Motor</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>NWJ76F</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Cadena</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>NWJ76F</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Freno delantero</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>NWJ76F</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Freno trasero</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>NWJ76F</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Pedal cambios</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>NWJ76F</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Embrague</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>NWJ76F</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Tablero</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Carlos Mario Osorio Taborda</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>NWJ76F</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Bocina</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>🟢 Bueno</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Sin observación</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>